<commit_message>
Update word and example listening instructions
</commit_message>
<xml_diff>
--- a/hsk1-vocabulary/HSK3.0_1급_유형별_QR단어장.xlsx
+++ b/hsk1-vocabulary/HSK3.0_1급_유형별_QR단어장.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="01_인사와 예절" sheetId="1" ns1:id="Rdf5484cba4a84819"/>
-    <sheet name="02_가족과 사람" sheetId="2" ns1:id="Rcf6c3228d60d41c4"/>
-    <sheet name="03_나와 너_가리키는 말" sheetId="3" ns1:id="R83dbb1594e26459d"/>
-    <sheet name="04_질문하는 말" sheetId="4" ns1:id="Ra510253c980c494e"/>
-    <sheet name="05_숫자와 수량" sheetId="5" ns1:id="Rb58e360f26504c80"/>
-    <sheet name="06_날짜와 시간" sheetId="6" ns1:id="R2d140205533f49af"/>
-    <sheet name="07_음식과 식사" sheetId="7" ns1:id="Rcfa6bca0f6c8402e"/>
-    <sheet name="08_집과 생활용품" sheetId="8" ns1:id="R99528257b6ed46cc"/>
-    <sheet name="09_장소와 교통" sheetId="9" ns1:id="R9e7c52fe40eb444a"/>
-    <sheet name="10_위치와 방향" sheetId="10" ns1:id="R158aadebe02b4cf5"/>
-    <sheet name="11_학교와 학습" sheetId="11" ns1:id="R3f8a345d6929470c"/>
-    <sheet name="12_일상과 활동" sheetId="12" ns1:id="R82d2e4142b424b7c"/>
-    <sheet name="13_생각과 감각" sheetId="13" ns1:id="Re9ad915fe9654a32"/>
-    <sheet name="14_상태와 평가" sheetId="14" ns1:id="R64c9ea6d3e71422b"/>
-    <sheet name="15_날씨_동물_건강" sheetId="15" ns1:id="Ra4a9c907a54d46b8"/>
-    <sheet name="16_문장을 잇는 말" sheetId="16" ns1:id="Re64975b2377e4614"/>
-    <sheet name="17_돈과 가격" sheetId="17" ns1:id="R20ab904407774026"/>
+    <sheet name="01_인사와 예절" sheetId="1" ns1:id="R17be673e8e014238"/>
+    <sheet name="02_가족과 사람" sheetId="2" ns1:id="Rd39178358dd54367"/>
+    <sheet name="03_나와 너_가리키는 말" sheetId="3" ns1:id="Ra5fd8f8ff3f34a41"/>
+    <sheet name="04_질문하는 말" sheetId="4" ns1:id="R93a3d5a5f6294324"/>
+    <sheet name="05_숫자와 수량" sheetId="5" ns1:id="Rd40368909fa547ca"/>
+    <sheet name="06_날짜와 시간" sheetId="6" ns1:id="R99d08b2428614894"/>
+    <sheet name="07_음식과 식사" sheetId="7" ns1:id="R87e77968a3f54e6a"/>
+    <sheet name="08_집과 생활용품" sheetId="8" ns1:id="R5925bb5c8a5f4067"/>
+    <sheet name="09_장소와 교통" sheetId="9" ns1:id="Re548293324874072"/>
+    <sheet name="10_위치와 방향" sheetId="10" ns1:id="Rf328ef39e009495e"/>
+    <sheet name="11_학교와 학습" sheetId="11" ns1:id="R3b359a26aae449bb"/>
+    <sheet name="12_일상과 활동" sheetId="12" ns1:id="R5b1840711e51479b"/>
+    <sheet name="13_생각과 감각" sheetId="13" ns1:id="R419554f2fbf74925"/>
+    <sheet name="14_상태와 평가" sheetId="14" ns1:id="R43a2ab120fd74318"/>
+    <sheet name="15_날씨_동물_건강" sheetId="15" ns1:id="R4d7549bac7214a6f"/>
+    <sheet name="16_문장을 잇는 말" sheetId="16" ns1:id="Rb3ab9dcc6ca143a1"/>
+    <sheet name="17_돈과 가격" sheetId="17" ns1:id="R28206fdcf6be4a8d"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'01_인사와 예절'!$A$1:$E$30</definedName>
@@ -250,13 +250,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="174e7bd3-059a-4109-9823-fb61f2d027fa"/>
+        <xdr:cNvPr id="1" name="29ad15b5-82cb-488d-b7ea-c9cfab06f491"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2e5dde96b9154155"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra183cf570fa04dd5"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -282,13 +282,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="a28ab884-3dec-47af-a0fa-262991b1ca1a"/>
+        <xdr:cNvPr id="1" name="5a382261-0e45-4669-b8b9-0429ea61a970"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0ed561e004a04c1e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R27516c672692403b"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -314,13 +314,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="2adf6068-87e6-4755-a603-8be703d2be62"/>
+        <xdr:cNvPr id="1" name="6f0816c4-c63f-4834-8af3-e00d837f47c8"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf74c1327b8334b46"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7b37a952c32e45bc"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -341,13 +341,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="1fb9ec5e-efb1-4c50-b14b-64fd8be083da"/>
+        <xdr:cNvPr id="2" name="319ceb17-b97c-4feb-8142-ab174619815e"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra6499b11dd6b4549"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4bf31b5a791d4434"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -373,13 +373,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="77397fec-68bc-4568-aae7-3b865a033a66"/>
+        <xdr:cNvPr id="1" name="849a703a-0b6a-4c1f-9285-7fe2274532d4"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rda6f387873f4436c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R86918acac6da4214"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -400,13 +400,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="0fc832c6-311e-450f-ab60-e086704a2dde"/>
+        <xdr:cNvPr id="2" name="21645b2b-0ba4-445c-b669-3089356abaf6"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R39fa5eef82da4aa3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc53b2ce4cf524b40"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -432,13 +432,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="b5378363-4edd-48fa-8c17-28fbb961fb90"/>
+        <xdr:cNvPr id="1" name="72d9dd28-a7c5-4ee1-a136-4c724ec0eb3c"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7623cd7a9b8743d0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4b8aef1a2f024040"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -464,13 +464,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="2a210aba-759a-4171-a86c-279e74e72b08"/>
+        <xdr:cNvPr id="1" name="db033d37-bbf4-4456-9dbe-ffe79238b0cd"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R778e19037f8f42cc"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R029bb7513d6541ba"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -496,13 +496,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="eaa0e2f4-ef25-40d5-acb6-890f715a9b41"/>
+        <xdr:cNvPr id="1" name="390f9c41-8944-4ce4-bf07-a28f6a0be63e"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R55d6c0bef3194655"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R75f80a6cb9984e64"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -528,13 +528,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="612eef2f-70db-4040-a376-c80ecf932800"/>
+        <xdr:cNvPr id="1" name="e952a2bb-64b4-4855-904e-8cd04f07d19b"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R138025849d5c43b7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4bf1487bd0fd40a4"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -555,13 +555,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="9736ac45-10b5-42c4-b19d-1f66c068c054"/>
+        <xdr:cNvPr id="2" name="820693c9-e09e-4c64-9f5c-82168cf18e01"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R05a28f27a99a4a13"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcc9bceb57be44083"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -587,13 +587,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="caa93cc3-bd5a-4319-a1ec-745bcc9a420f"/>
+        <xdr:cNvPr id="1" name="bdb39616-62c6-475a-be94-b70007f80741"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9a4a4dbec9314977"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd9dfa2fb9a4c43b7"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -619,13 +619,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="a7aa90ec-45af-44f7-bb8f-865e714b0922"/>
+        <xdr:cNvPr id="1" name="05265d91-a579-4955-9478-3976a2ad8bd6"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0f503a93c45c4ab5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Redb9c72fee6a405e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -646,13 +646,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="96dd0376-c1b7-47d8-a740-79bc5a8969e5"/>
+        <xdr:cNvPr id="2" name="ec8f2416-b235-475a-9e5a-1dfb61593917"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbde493b22b624f95"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9880fa7dcb5945e8"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -678,13 +678,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="c121ee4f-8a73-4b33-a3bb-f3c4ae0918c6"/>
+        <xdr:cNvPr id="1" name="5c1626fa-0235-4fc6-b198-d91ea4a09be7"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc5a77612a4574f47"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R73493d98fe334745"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -705,13 +705,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="bbab629d-ace3-45ac-873a-eecb80f0c0c4"/>
+        <xdr:cNvPr id="2" name="0090619a-2386-406d-86b3-27d03df4e745"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rff31048108d14431"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9afbb76bd8d747e0"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -737,13 +737,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="f78c2604-8995-41ac-b031-b263fda4a41d"/>
+        <xdr:cNvPr id="1" name="c3295ced-7a5a-4e9b-bb47-7cf6630ac282"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3b1b5cf017c440ea"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdf80dcbad4ef4454"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -769,13 +769,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="1ff36c22-756e-41a6-93c1-c8815cee4718"/>
+        <xdr:cNvPr id="1" name="ee15cbad-7802-43df-95d7-0d7e975f1e51"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R06a2bb6f787a4adb"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R22f3064f66944120"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -796,13 +796,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="0f298ea6-fbe9-4241-a217-d31bcf22974f"/>
+        <xdr:cNvPr id="2" name="e0afd668-bad0-4189-9935-c9419a36efcf"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rfa425e8a16064da2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2f788de7b8e646d3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -828,13 +828,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="f965fd21-7f32-4d24-9664-7aaa479e1802"/>
+        <xdr:cNvPr id="1" name="dd348c26-1a05-4214-bf15-eee13bcdc80f"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf72a6fc2b26d4852"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R018d6ab8c6b04432"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -855,13 +855,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="0df1583a-131a-4818-aa52-1a561934af10"/>
+        <xdr:cNvPr id="2" name="84e7974b-bbde-4937-ba7f-cc77de5f655b"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb6e0a4f0f8884315"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R614defb533ea4d73"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -887,13 +887,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="0758186c-a22e-4fff-8561-7c88f83645b9"/>
+        <xdr:cNvPr id="1" name="40cf9d22-25b9-46d1-99de-7f91cb8e2681"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6b6b533b0b2f425a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc4bc72a9064f4be2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -914,13 +914,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="579e9ae0-f4a6-4eb7-8784-ffbe3c6cd96b"/>
+        <xdr:cNvPr id="2" name="4df4f486-1a86-4bb0-8e4b-252df29e325e"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R01b9986c602941a1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R13d7db85f356490a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -946,13 +946,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="ae9728a1-3409-4cc5-8d2c-2e373750f9fb"/>
+        <xdr:cNvPr id="1" name="fd2378ad-3698-4755-90e1-f6628b328a4c"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R54bef92481a74580"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7eec169e13a140a2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -978,13 +978,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="b21babcf-4337-4986-b672-2e8c74c7aa96"/>
+        <xdr:cNvPr id="1" name="1fe5429a-ea82-4252-9da7-73b1e3d13b12"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R51abbe26fa434ca2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rad7a5d4f13834956"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1005,13 +1005,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="efce6014-71b1-41a3-9e83-dc42f0dabed5"/>
+        <xdr:cNvPr id="2" name="23db6176-4ef2-44fd-96cd-678f6e8b3f1e"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R73c8196b50f44c07"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2e76bd22664e4901"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1283,7 +1283,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1579,7 +1579,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="R6910e0195b374ebb"/>
+  <drawing ns1:id="Rcc0fd9f133d34713"/>
 </worksheet>
 </file>
 
@@ -1650,7 +1650,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1926,7 +1926,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="Rd99e2e1c76a64eb2"/>
+  <drawing ns1:id="R350c5897c75f4d37"/>
 </worksheet>
 </file>
 
@@ -1997,7 +1997,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -2353,7 +2353,7 @@
     </row>
     <row r="37" ht="12" customHeight="1">
       <c r="A37" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -2689,7 +2689,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="Reb64ba0b90944d1e"/>
+  <drawing ns1:id="Rc4fd01417e5246ef"/>
 </worksheet>
 </file>
 
@@ -2760,7 +2760,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -3126,7 +3126,7 @@
     </row>
     <row r="37" ht="12" customHeight="1">
       <c r="A37" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -3472,7 +3472,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="R74628bda69c44c2f"/>
+  <drawing ns1:id="R6e38087925514c98"/>
 </worksheet>
 </file>
 
@@ -3543,7 +3543,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -3849,7 +3849,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="Rab13033004874542"/>
+  <drawing ns1:id="Rf18e146b96a54391"/>
 </worksheet>
 </file>
 
@@ -3920,7 +3920,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -4256,7 +4256,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="Rcbd92b905db347df"/>
+  <drawing ns1:id="Rc879aa12ba914c0e"/>
 </worksheet>
 </file>
 
@@ -4327,7 +4327,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -4643,7 +4643,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="R257e6b8dca104044"/>
+  <drawing ns1:id="Rb813600eca6e40c2"/>
 </worksheet>
 </file>
 
@@ -4714,7 +4714,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -5080,7 +5080,7 @@
     </row>
     <row r="37" ht="12" customHeight="1">
       <c r="A37" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -5416,7 +5416,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="Rb91191925274463b"/>
+  <drawing ns1:id="R787836ff6e8242f4"/>
 </worksheet>
 </file>
 
@@ -5487,7 +5487,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -5713,7 +5713,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="Racde18d7b59743f2"/>
+  <drawing ns1:id="R6125841fbe0d4403"/>
 </worksheet>
 </file>
 
@@ -5784,7 +5784,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -6120,7 +6120,7 @@
     </row>
     <row r="37" ht="12" customHeight="1">
       <c r="A37" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -6436,7 +6436,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="R34dd4f4c9efc46eb"/>
+  <drawing ns1:id="R5b7599a38a6940a8"/>
 </worksheet>
 </file>
 
@@ -6507,7 +6507,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -6863,7 +6863,7 @@
     </row>
     <row r="37" ht="12" customHeight="1">
       <c r="A37" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -7199,7 +7199,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="R8dd60bb20e384436"/>
+  <drawing ns1:id="R47629859d5434873"/>
 </worksheet>
 </file>
 
@@ -7270,7 +7270,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -7576,7 +7576,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="R28797f20f3af4a50"/>
+  <drawing ns1:id="R45adf840a37d4bfe"/>
 </worksheet>
 </file>
 
@@ -7647,7 +7647,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -8023,7 +8023,7 @@
     </row>
     <row r="37" ht="12" customHeight="1">
       <c r="A37" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -8379,7 +8379,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="Rd16fd4dc0af5436c"/>
+  <drawing ns1:id="Rf7635aeeff2246b6"/>
 </worksheet>
 </file>
 
@@ -8450,7 +8450,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -8826,7 +8826,7 @@
     </row>
     <row r="37" ht="12" customHeight="1">
       <c r="A37" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -9172,7 +9172,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="R521ac7b1f4714a5b"/>
+  <drawing ns1:id="R716f3e5449644972"/>
 </worksheet>
 </file>
 
@@ -9243,7 +9243,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -9579,7 +9579,7 @@
     </row>
     <row r="37" ht="12" customHeight="1">
       <c r="A37" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -9885,7 +9885,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="Rceddaf11441842f2"/>
+  <drawing ns1:id="R0d6d692c3ae544c8"/>
 </worksheet>
 </file>
 
@@ -9956,7 +9956,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -10262,7 +10262,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="R8a56957ae16c48f0"/>
+  <drawing ns1:id="R7815877af2734c59"/>
 </worksheet>
 </file>
 
@@ -10333,7 +10333,7 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -10659,7 +10659,7 @@
     </row>
     <row r="37" ht="12" customHeight="1">
       <c r="A37" s="6" t="str">
-        <v>이 페이지의 단어만 중국어로 두 번씩 읽습니다.</v>
+        <v>단어 두 번, 예문 한 번 순서로 읽습니다.</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -10965,6 +10965,6 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="R270ae8d473ef4e1f"/>
+  <drawing ns1:id="R4cb1d49b5dc84a6d"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Review HSK 1 words and correct wei pinyin and xia meaning
</commit_message>
<xml_diff>
--- a/hsk1-vocabulary/HSK3.0_1급_유형별_QR단어장.xlsx
+++ b/hsk1-vocabulary/HSK3.0_1급_유형별_QR단어장.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="01_인사와 예절" sheetId="1" ns1:id="R17be673e8e014238"/>
-    <sheet name="02_가족과 사람" sheetId="2" ns1:id="Rd39178358dd54367"/>
-    <sheet name="03_나와 너_가리키는 말" sheetId="3" ns1:id="Ra5fd8f8ff3f34a41"/>
-    <sheet name="04_질문하는 말" sheetId="4" ns1:id="R93a3d5a5f6294324"/>
-    <sheet name="05_숫자와 수량" sheetId="5" ns1:id="Rd40368909fa547ca"/>
-    <sheet name="06_날짜와 시간" sheetId="6" ns1:id="R99d08b2428614894"/>
-    <sheet name="07_음식과 식사" sheetId="7" ns1:id="R87e77968a3f54e6a"/>
-    <sheet name="08_집과 생활용품" sheetId="8" ns1:id="R5925bb5c8a5f4067"/>
-    <sheet name="09_장소와 교통" sheetId="9" ns1:id="Re548293324874072"/>
-    <sheet name="10_위치와 방향" sheetId="10" ns1:id="Rf328ef39e009495e"/>
-    <sheet name="11_학교와 학습" sheetId="11" ns1:id="R3b359a26aae449bb"/>
-    <sheet name="12_일상과 활동" sheetId="12" ns1:id="R5b1840711e51479b"/>
-    <sheet name="13_생각과 감각" sheetId="13" ns1:id="R419554f2fbf74925"/>
-    <sheet name="14_상태와 평가" sheetId="14" ns1:id="R43a2ab120fd74318"/>
-    <sheet name="15_날씨_동물_건강" sheetId="15" ns1:id="R4d7549bac7214a6f"/>
-    <sheet name="16_문장을 잇는 말" sheetId="16" ns1:id="Rb3ab9dcc6ca143a1"/>
-    <sheet name="17_돈과 가격" sheetId="17" ns1:id="R28206fdcf6be4a8d"/>
+    <sheet name="01_인사와 예절" sheetId="1" ns1:id="Rfeafdaa83c5841c8"/>
+    <sheet name="02_가족과 사람" sheetId="2" ns1:id="R1eff8952b8e343fa"/>
+    <sheet name="03_나와 너_가리키는 말" sheetId="3" ns1:id="R8d8e8a56662f4470"/>
+    <sheet name="04_질문하는 말" sheetId="4" ns1:id="R5298b34fcdef44c1"/>
+    <sheet name="05_숫자와 수량" sheetId="5" ns1:id="Rc3863187e4024ed9"/>
+    <sheet name="06_날짜와 시간" sheetId="6" ns1:id="R1a9e360e4b85400d"/>
+    <sheet name="07_음식과 식사" sheetId="7" ns1:id="R18043be64a344c47"/>
+    <sheet name="08_집과 생활용품" sheetId="8" ns1:id="R1d828cf9716744b4"/>
+    <sheet name="09_장소와 교통" sheetId="9" ns1:id="R1baf3081da824179"/>
+    <sheet name="10_위치와 방향" sheetId="10" ns1:id="R0d12cbcbe0544668"/>
+    <sheet name="11_학교와 학습" sheetId="11" ns1:id="Rc8d77830cb86475a"/>
+    <sheet name="12_일상과 활동" sheetId="12" ns1:id="R2c657d48bbff49b9"/>
+    <sheet name="13_생각과 감각" sheetId="13" ns1:id="Re633a40d8ee445c8"/>
+    <sheet name="14_상태와 평가" sheetId="14" ns1:id="R216f14516f7f431e"/>
+    <sheet name="15_날씨_동물_건강" sheetId="15" ns1:id="R7b673fecb26c41c8"/>
+    <sheet name="16_문장을 잇는 말" sheetId="16" ns1:id="Rf03e419b9b7d4652"/>
+    <sheet name="17_돈과 가격" sheetId="17" ns1:id="Rf05cf3e9bbe84115"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'01_인사와 예절'!$A$1:$E$30</definedName>
@@ -250,13 +250,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="29ad15b5-82cb-488d-b7ea-c9cfab06f491"/>
+        <xdr:cNvPr id="1" name="7ea9efa3-66a7-4cef-b6d0-5365095e9ff8"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra183cf570fa04dd5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9604a134c6bf4b02"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -282,13 +282,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="5a382261-0e45-4669-b8b9-0429ea61a970"/>
+        <xdr:cNvPr id="1" name="ced78a21-4314-4f77-87a4-641e6fe281eb"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R27516c672692403b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R188819c1c8154b8e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -314,13 +314,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="6f0816c4-c63f-4834-8af3-e00d837f47c8"/>
+        <xdr:cNvPr id="1" name="cb293caf-5c23-4961-9cc8-2a222857b9e9"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7b37a952c32e45bc"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra9d94d64cd88493d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -341,13 +341,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="319ceb17-b97c-4feb-8142-ab174619815e"/>
+        <xdr:cNvPr id="2" name="82b42d4e-f913-44d5-aedc-a236799f517c"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4bf31b5a791d4434"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re8dbb3d9aa8b43ad"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -373,13 +373,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="849a703a-0b6a-4c1f-9285-7fe2274532d4"/>
+        <xdr:cNvPr id="1" name="448b7670-375e-49ae-8d63-478e11d3ce84"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R86918acac6da4214"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5c3f3d9e13f04a35"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -400,13 +400,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="21645b2b-0ba4-445c-b669-3089356abaf6"/>
+        <xdr:cNvPr id="2" name="465599c7-758a-48d0-8d9f-211b195d8bae"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc53b2ce4cf524b40"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R420adf5865ef4c31"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -432,13 +432,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="72d9dd28-a7c5-4ee1-a136-4c724ec0eb3c"/>
+        <xdr:cNvPr id="1" name="8b445caf-bbec-4234-ab71-6996b7ccb0b1"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4b8aef1a2f024040"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R48b8ca09795e478c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -464,13 +464,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="db033d37-bbf4-4456-9dbe-ffe79238b0cd"/>
+        <xdr:cNvPr id="1" name="9d99a0b8-f4c6-484b-b505-d044aec95fa1"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R029bb7513d6541ba"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra3f3ff15cbc34163"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -496,13 +496,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="390f9c41-8944-4ce4-bf07-a28f6a0be63e"/>
+        <xdr:cNvPr id="1" name="dff7fee5-5481-4aa5-8a23-14f72b6338d2"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R75f80a6cb9984e64"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0ff0af41b8bb48fb"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -528,13 +528,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="e952a2bb-64b4-4855-904e-8cd04f07d19b"/>
+        <xdr:cNvPr id="1" name="03efd536-0d1a-435a-b6ba-847c9bebad26"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4bf1487bd0fd40a4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Raacf9859817c4009"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -555,13 +555,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="820693c9-e09e-4c64-9f5c-82168cf18e01"/>
+        <xdr:cNvPr id="2" name="3d4c2540-ba2d-406f-8b2d-8613174f6f34"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcc9bceb57be44083"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6db3fda75e57438a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -587,13 +587,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="bdb39616-62c6-475a-be94-b70007f80741"/>
+        <xdr:cNvPr id="1" name="da416006-7994-421f-b1e8-789f16901c65"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd9dfa2fb9a4c43b7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3c598361c2364281"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -619,13 +619,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="05265d91-a579-4955-9478-3976a2ad8bd6"/>
+        <xdr:cNvPr id="1" name="9a362586-0c08-428a-9e33-66a5fa343bdd"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Redb9c72fee6a405e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0876566dc6064cb2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -646,13 +646,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="ec8f2416-b235-475a-9e5a-1dfb61593917"/>
+        <xdr:cNvPr id="2" name="72931b67-6c82-4b88-8d3e-21e88624fe78"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9880fa7dcb5945e8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7210e0c1b39043bb"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -678,13 +678,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="5c1626fa-0235-4fc6-b198-d91ea4a09be7"/>
+        <xdr:cNvPr id="1" name="f5634241-1045-436e-a911-b9778d3a8f93"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R73493d98fe334745"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rad7aa739c83d44eb"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -705,13 +705,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="0090619a-2386-406d-86b3-27d03df4e745"/>
+        <xdr:cNvPr id="2" name="66507ba7-6c03-4a24-8764-db7b67efe95e"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9afbb76bd8d747e0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcbf1707a74f24415"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -737,13 +737,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="c3295ced-7a5a-4e9b-bb47-7cf6630ac282"/>
+        <xdr:cNvPr id="1" name="55bbd28f-436c-4537-80ad-dcfdbf03db09"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdf80dcbad4ef4454"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R694d61defd084c1c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -769,13 +769,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="ee15cbad-7802-43df-95d7-0d7e975f1e51"/>
+        <xdr:cNvPr id="1" name="fdc15341-8d70-43a9-9bfd-21d7345bf649"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R22f3064f66944120"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8a294b0758924185"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -796,13 +796,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="e0afd668-bad0-4189-9935-c9419a36efcf"/>
+        <xdr:cNvPr id="2" name="61d2577c-3d95-45ae-b781-3d178bdc17c1"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2f788de7b8e646d3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc83b1e3494754069"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -828,13 +828,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="dd348c26-1a05-4214-bf15-eee13bcdc80f"/>
+        <xdr:cNvPr id="1" name="b4552391-6bdf-4039-8b9d-1d6157cfeefd"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R018d6ab8c6b04432"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2b141e76c99243ce"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -855,13 +855,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="84e7974b-bbde-4937-ba7f-cc77de5f655b"/>
+        <xdr:cNvPr id="2" name="2b4a2970-a733-4e12-baa9-5381732ab5fa"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R614defb533ea4d73"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2fd6c3002a6d4225"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -887,13 +887,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="40cf9d22-25b9-46d1-99de-7f91cb8e2681"/>
+        <xdr:cNvPr id="1" name="7e4e591c-90b9-48cc-a1ad-70dde25c463b"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc4bc72a9064f4be2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R820fae82caae439e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -914,13 +914,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="4df4f486-1a86-4bb0-8e4b-252df29e325e"/>
+        <xdr:cNvPr id="2" name="69703a31-685f-4424-bcd6-c61cfca7ee7b"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R13d7db85f356490a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R61e2a86d3ae348e2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -946,13 +946,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="fd2378ad-3698-4755-90e1-f6628b328a4c"/>
+        <xdr:cNvPr id="1" name="e8f1bfc7-b521-4b83-a072-74cd7c55307d"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7eec169e13a140a2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbb9d3033f20f4c00"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -978,13 +978,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="1fe5429a-ea82-4252-9da7-73b1e3d13b12"/>
+        <xdr:cNvPr id="1" name="fa33ca2a-b556-4acf-98c2-240e686b0c77"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rad7a5d4f13834956"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R010e24602896492f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1005,13 +1005,13 @@
     <xdr:ext cx="1257300" cy="1257300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="23db6176-4ef2-44fd-96cd-678f6e8b3f1e"/>
+        <xdr:cNvPr id="2" name="1ae04549-47f4-4e3d-bd66-ff7c24e6fe38"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2e76bd22664e4901"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R557d7abf993a47d7"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1441,7 +1441,7 @@
         <v>喂1</v>
       </c>
       <c r="C17" s="26" t="str">
-        <v>wèi</v>
+        <v>wéi</v>
       </c>
       <c r="D17" s="27" t="str">
         <v>여보세요</v>
@@ -1544,7 +1544,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -1579,7 +1579,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="Rcc0fd9f133d34713"/>
+  <drawing ns1:id="Ra06d0886159c4242"/>
 </worksheet>
 </file>
 
@@ -1811,7 +1811,7 @@
         <v>xià</v>
       </c>
       <c r="D17" s="27" t="str">
-        <v>아래 / 내리다, 타다 / 번(양사)</v>
+        <v>아래 / 내리다 / 번(양사)</v>
       </c>
       <c r="E17" s="28" t="str">
         <v>我在楼下等你。</v>
@@ -1891,7 +1891,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -1926,7 +1926,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="R350c5897c75f4d37"/>
+  <drawing ns1:id="R55e5804581a349c8"/>
 </worksheet>
 </file>
 
@@ -2278,7 +2278,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -2644,7 +2644,7 @@
     </row>
     <row r="58" ht="12" customHeight="1">
       <c r="A58" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B58" s="29"/>
       <c r="C58" s="29"/>
@@ -2689,7 +2689,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="Rc4fd01417e5246ef"/>
+  <drawing ns1:id="R1777b3c95498433c"/>
 </worksheet>
 </file>
 
@@ -3051,7 +3051,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -3427,7 +3427,7 @@
     </row>
     <row r="58" ht="12" customHeight="1">
       <c r="A58" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B58" s="29"/>
       <c r="C58" s="29"/>
@@ -3472,7 +3472,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="R6e38087925514c98"/>
+  <drawing ns1:id="R24f4938d45ca4c79"/>
 </worksheet>
 </file>
 
@@ -3814,7 +3814,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -3849,7 +3849,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="Rf18e146b96a54391"/>
+  <drawing ns1:id="R56bb0da38e6e4111"/>
 </worksheet>
 </file>
 
@@ -4221,7 +4221,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -4256,7 +4256,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="Rc879aa12ba914c0e"/>
+  <drawing ns1:id="Rff4b2542cb774925"/>
 </worksheet>
 </file>
 
@@ -4608,7 +4608,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -4643,7 +4643,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="Rb813600eca6e40c2"/>
+  <drawing ns1:id="Rf2c42568790b4a57"/>
 </worksheet>
 </file>
 
@@ -5005,7 +5005,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -5371,7 +5371,7 @@
     </row>
     <row r="58" ht="12" customHeight="1">
       <c r="A58" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B58" s="29"/>
       <c r="C58" s="29"/>
@@ -5416,7 +5416,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="R787836ff6e8242f4"/>
+  <drawing ns1:id="R7f00b93e1ab443d7"/>
 </worksheet>
 </file>
 
@@ -5678,7 +5678,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -5713,7 +5713,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="R6125841fbe0d4403"/>
+  <drawing ns1:id="R41e0246e57974522"/>
 </worksheet>
 </file>
 
@@ -6045,7 +6045,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -6391,7 +6391,7 @@
     </row>
     <row r="58" ht="12" customHeight="1">
       <c r="A58" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B58" s="29"/>
       <c r="C58" s="29"/>
@@ -6436,7 +6436,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="R5b7599a38a6940a8"/>
+  <drawing ns1:id="R6f03ac660879402b"/>
 </worksheet>
 </file>
 
@@ -6788,7 +6788,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -7154,7 +7154,7 @@
     </row>
     <row r="58" ht="12" customHeight="1">
       <c r="A58" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B58" s="29"/>
       <c r="C58" s="29"/>
@@ -7199,7 +7199,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="R47629859d5434873"/>
+  <drawing ns1:id="R4ce1bf223c7d43c6"/>
 </worksheet>
 </file>
 
@@ -7541,7 +7541,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -7576,7 +7576,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="R45adf840a37d4bfe"/>
+  <drawing ns1:id="R38b9b02ab2974401"/>
 </worksheet>
 </file>
 
@@ -7948,7 +7948,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -8334,7 +8334,7 @@
     </row>
     <row r="58" ht="12" customHeight="1">
       <c r="A58" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B58" s="29"/>
       <c r="C58" s="29"/>
@@ -8379,7 +8379,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="Rf7635aeeff2246b6"/>
+  <drawing ns1:id="Rdea4b59dc49a4fe8"/>
 </worksheet>
 </file>
 
@@ -8751,7 +8751,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -9127,7 +9127,7 @@
     </row>
     <row r="58" ht="12" customHeight="1">
       <c r="A58" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B58" s="29"/>
       <c r="C58" s="29"/>
@@ -9172,7 +9172,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="R716f3e5449644972"/>
+  <drawing ns1:id="Rd285e605e24d4980"/>
 </worksheet>
 </file>
 
@@ -9504,7 +9504,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -9840,7 +9840,7 @@
     </row>
     <row r="58" ht="12" customHeight="1">
       <c r="A58" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B58" s="29"/>
       <c r="C58" s="29"/>
@@ -9885,7 +9885,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="R0d6d692c3ae544c8"/>
+  <drawing ns1:id="Rd2b7e1e0c805479c"/>
 </worksheet>
 </file>
 
@@ -10227,7 +10227,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -10262,7 +10262,7 @@
   </mergeCells>
   <pageMargins left="0.33" right="0.33" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
-  <drawing ns1:id="R7815877af2734c59"/>
+  <drawing ns1:id="R43b335ac04964772"/>
 </worksheet>
 </file>
 
@@ -10584,7 +10584,7 @@
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -10920,7 +10920,7 @@
     </row>
     <row r="58" ht="12" customHeight="1">
       <c r="A58" s="29" t="str">
-        <v>원본 300단어의 병음·뜻·예문 유지 / 중국어 합성음성</v>
+        <v>300개 단어 / 병음·뜻 재점검 / 중국어 합성음성</v>
       </c>
       <c r="B58" s="29"/>
       <c r="C58" s="29"/>
@@ -10965,6 +10965,6 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="30" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing ns1:id="R4cb1d49b5dc84a6d"/>
+  <drawing ns1:id="R0851dc2e652e4294"/>
 </worksheet>
 </file>
</xml_diff>